<commit_message>
Pipeline live (real funnel); outreach tool creates Gmail drafts; 3 creators -> Outreached
</commit_message>
<xml_diff>
--- a/workers/Simify_YouTube_MicroNano_Prospects.xlsx
+++ b/workers/Simify_YouTube_MicroNano_Prospects.xlsx
@@ -1084,7 +1084,7 @@
       </c>
       <c r="K10" s="6" t="inlineStr">
         <is>
-          <t>Not contacted</t>
+          <t>Contacted</t>
         </is>
       </c>
       <c r="L10" s="6" t="inlineStr"/>
@@ -1722,7 +1722,7 @@
       </c>
       <c r="K21" s="6" t="inlineStr">
         <is>
-          <t>Not contacted</t>
+          <t>Contacted</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr"/>
@@ -2186,7 +2186,7 @@
       </c>
       <c r="K29" s="3" t="inlineStr">
         <is>
-          <t>Not contacted</t>
+          <t>Contacted</t>
         </is>
       </c>
       <c r="L29" s="3" t="inlineStr"/>
@@ -7987,10 +7987,7 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr"/>
-      <c r="B3" t="inlineStr"/>
-    </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
@@ -8022,10 +8019,7 @@
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr"/>
-      <c r="B7" t="inlineStr"/>
-    </row>
+    <row r="7"/>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
@@ -8081,10 +8075,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
-    </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>

</xml_diff>